<commit_message>
Update chess menu research spreadsheet
</commit_message>
<xml_diff>
--- a/research/chess_menu_research.xlsx
+++ b/research/chess_menu_research.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ajin/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ajin/Documents/GitHub/dsc-website-spec/research/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55DC7387-0113-EA4B-BB5B-17539B42311D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9656FCB5-DDCF-7F47-9E57-1E82E8D39F94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1598,7 +1598,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1614,19 +1614,6 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="9"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -1636,8 +1623,15 @@
       <name val="Consolas"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1646,22 +1640,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F3864"/>
+        <fgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9E1F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF2F5496"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFCE4D6"/>
+        <fgColor theme="3"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1716,32 +1701,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2051,1137 +2033,1137 @@
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="25" width="42" customWidth="1"/>
-    <col min="26" max="28" width="30" customWidth="1"/>
+    <col min="26" max="28" width="30" hidden="1" customWidth="1"/>
     <col min="29" max="48" width="42" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:48" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="7"/>
+      <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="V1" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="W1" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="X1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Y1" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="Z1" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AA1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AB1" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AC1" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AD1" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AE1" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AF1" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AG1" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AH1" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AI1" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AJ1" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AK1" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AL1" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="AM1" s="2" t="s">
+      <c r="AM1" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="AN1" s="2" t="s">
+      <c r="AN1" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="AO1" s="2" t="s">
+      <c r="AO1" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="AP1" s="2" t="s">
+      <c r="AP1" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="AQ1" s="2" t="s">
+      <c r="AQ1" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="AR1" s="2" t="s">
+      <c r="AR1" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="AS1" s="2" t="s">
+      <c r="AS1" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="AT1" s="2" t="s">
+      <c r="AT1" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="AU1" s="2" t="s">
+      <c r="AU1" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="AV1" s="2" t="s">
+      <c r="AV1" s="8" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="P2" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="Q2" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="R2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="S2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="T2" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="U2" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="V2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="W2" s="4" t="s">
+      <c r="W2" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="X2" s="4" t="s">
+      <c r="X2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="Y2" s="4" t="s">
+      <c r="Y2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="Z2" s="7" t="s">
+      <c r="Z2" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="AA2" s="7" t="s">
+      <c r="AA2" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="AB2" s="7" t="s">
+      <c r="AB2" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="AC2" s="4" t="s">
+      <c r="AC2" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="AD2" s="4" t="s">
+      <c r="AD2" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="AE2" s="4" t="s">
+      <c r="AE2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AF2" s="4" t="s">
+      <c r="AF2" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="AG2" s="4" t="s">
+      <c r="AG2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AH2" s="4" t="s">
+      <c r="AH2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AI2" s="4" t="s">
+      <c r="AI2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AJ2" s="4" t="s">
+      <c r="AJ2" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="AK2" s="4" t="s">
+      <c r="AK2" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="AL2" s="4" t="s">
+      <c r="AL2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AM2" s="4" t="s">
+      <c r="AM2" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="AN2" s="4" t="s">
+      <c r="AN2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AO2" s="4" t="s">
+      <c r="AO2" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="AP2" s="4" t="s">
+      <c r="AP2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="AQ2" s="4" t="s">
+      <c r="AQ2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AR2" s="4" t="s">
+      <c r="AR2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AS2" s="4" t="s">
+      <c r="AS2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="AT2" s="4" t="s">
+      <c r="AT2" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="AU2" s="4" t="s">
+      <c r="AU2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AV2" s="4" t="s">
+      <c r="AV2" s="1" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="J3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="L3" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="M3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="N3" s="4" t="s">
+      <c r="N3" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="O3" s="4" t="s">
+      <c r="O3" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="P3" s="4" t="s">
+      <c r="P3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="Q3" s="4" t="s">
+      <c r="Q3" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="R3" s="4" t="s">
+      <c r="R3" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="S3" s="4" t="s">
+      <c r="S3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="T3" s="4" t="s">
+      <c r="T3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U3" s="4" t="s">
+      <c r="U3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="V3" s="4" t="s">
+      <c r="V3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="W3" s="4" t="s">
+      <c r="W3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="X3" s="4" t="s">
+      <c r="X3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="Y3" s="4" t="s">
+      <c r="Y3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="Z3" s="8"/>
-      <c r="AA3" s="8"/>
-      <c r="AB3" s="8"/>
-      <c r="AC3" s="4" t="s">
+      <c r="Z3" s="5"/>
+      <c r="AA3" s="5"/>
+      <c r="AB3" s="5"/>
+      <c r="AC3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="AD3" s="4" t="s">
+      <c r="AD3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AE3" s="4" t="s">
+      <c r="AE3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AF3" s="4" t="s">
+      <c r="AF3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AG3" s="4" t="s">
+      <c r="AG3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="AH3" s="4" t="s">
+      <c r="AH3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AI3" s="4" t="s">
+      <c r="AI3" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="AJ3" s="4" t="s">
+      <c r="AJ3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AK3" s="4" t="s">
+      <c r="AK3" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="AL3" s="4" t="s">
+      <c r="AL3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AM3" s="4" t="s">
+      <c r="AM3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="AN3" s="4" t="s">
+      <c r="AN3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AO3" s="4" t="s">
+      <c r="AO3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AP3" s="4" t="s">
+      <c r="AP3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AQ3" s="4" t="s">
+      <c r="AQ3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="AR3" s="4" t="s">
+      <c r="AR3" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="AS3" s="4" t="s">
+      <c r="AS3" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="AT3" s="4" t="s">
+      <c r="AT3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AU3" s="4" t="s">
+      <c r="AU3" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="AV3" s="4" t="s">
+      <c r="AV3" s="1" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:48" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="J4" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="K4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="L4" s="5" t="s">
+      <c r="L4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="M4" s="5" t="s">
+      <c r="M4" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="N4" s="5" t="s">
+      <c r="N4" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="O4" s="5" t="s">
+      <c r="O4" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="P4" s="5" t="s">
+      <c r="P4" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="Q4" s="5" t="s">
+      <c r="Q4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="R4" s="5" t="s">
+      <c r="R4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="S4" s="5" t="s">
+      <c r="S4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="T4" s="5" t="s">
+      <c r="T4" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="U4" s="5" t="s">
+      <c r="U4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="V4" s="5" t="s">
+      <c r="V4" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="W4" s="5" t="s">
+      <c r="W4" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="X4" s="5" t="s">
+      <c r="X4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="Y4" s="5" t="s">
+      <c r="Y4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="Z4" s="8"/>
-      <c r="AA4" s="8"/>
-      <c r="AB4" s="8"/>
-      <c r="AC4" s="5" t="s">
+      <c r="Z4" s="5"/>
+      <c r="AA4" s="5"/>
+      <c r="AB4" s="5"/>
+      <c r="AC4" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AD4" s="5" t="s">
+      <c r="AD4" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="AE4" s="5" t="s">
+      <c r="AE4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="AF4" s="5" t="s">
+      <c r="AF4" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="AG4" s="5" t="s">
+      <c r="AG4" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AH4" s="5" t="s">
+      <c r="AH4" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="AI4" s="5" t="s">
+      <c r="AI4" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="AJ4" s="5" t="s">
+      <c r="AJ4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="AK4" s="5" t="s">
+      <c r="AK4" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="AL4" s="5" t="s">
+      <c r="AL4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="AM4" s="5" t="s">
+      <c r="AM4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="AN4" s="5" t="s">
+      <c r="AN4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="AO4" s="5" t="s">
+      <c r="AO4" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="AP4" s="5" t="s">
+      <c r="AP4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="AQ4" s="5" t="s">
+      <c r="AQ4" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="AR4" s="5" t="s">
+      <c r="AR4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="AS4" s="5" t="s">
+      <c r="AS4" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="AT4" s="5" t="s">
+      <c r="AT4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="AU4" s="5" t="s">
+      <c r="AU4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="AV4" s="5" t="s">
+      <c r="AV4" s="2" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:48" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="J5" s="5" t="s">
+      <c r="J5" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="K5" s="5" t="s">
+      <c r="K5" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="L5" s="5" t="s">
+      <c r="L5" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="M5" s="5" t="s">
+      <c r="M5" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="N5" s="5" t="s">
+      <c r="N5" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="O5" s="5" t="s">
+      <c r="O5" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="P5" s="5" t="s">
+      <c r="P5" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="Q5" s="5" t="s">
+      <c r="Q5" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="R5" s="5" t="s">
+      <c r="R5" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="S5" s="5" t="s">
+      <c r="S5" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="T5" s="5" t="s">
+      <c r="T5" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="U5" s="5" t="s">
+      <c r="U5" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="V5" s="5" t="s">
+      <c r="V5" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="W5" s="5" t="s">
+      <c r="W5" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="X5" s="5" t="s">
+      <c r="X5" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="Y5" s="5" t="s">
+      <c r="Y5" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="Z5" s="8"/>
-      <c r="AA5" s="8"/>
-      <c r="AB5" s="8"/>
-      <c r="AC5" s="5" t="s">
+      <c r="Z5" s="5"/>
+      <c r="AA5" s="5"/>
+      <c r="AB5" s="5"/>
+      <c r="AC5" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="AD5" s="5" t="s">
+      <c r="AD5" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="AE5" s="5" t="s">
+      <c r="AE5" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="AF5" s="5" t="s">
+      <c r="AF5" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="AG5" s="5" t="s">
+      <c r="AG5" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="AH5" s="5" t="s">
+      <c r="AH5" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="AI5" s="5" t="s">
+      <c r="AI5" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="AJ5" s="5" t="s">
+      <c r="AJ5" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="AK5" s="5" t="s">
+      <c r="AK5" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="AL5" s="5" t="s">
+      <c r="AL5" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="AM5" s="5" t="s">
+      <c r="AM5" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="AN5" s="5" t="s">
+      <c r="AN5" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="AO5" s="5" t="s">
+      <c r="AO5" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="AP5" s="5" t="s">
+      <c r="AP5" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="AQ5" s="5" t="s">
+      <c r="AQ5" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="AR5" s="5" t="s">
+      <c r="AR5" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="AS5" s="5" t="s">
+      <c r="AS5" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="AT5" s="5" t="s">
+      <c r="AT5" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="AU5" s="5" t="s">
+      <c r="AU5" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="AV5" s="5" t="s">
+      <c r="AV5" s="2" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="6" spans="1:48" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="J6" s="5" t="s">
+      <c r="J6" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="K6" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="L6" s="5" t="s">
+      <c r="L6" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="M6" s="5" t="s">
+      <c r="M6" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="N6" s="5" t="s">
+      <c r="N6" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="O6" s="5" t="s">
+      <c r="O6" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="P6" s="5" t="s">
+      <c r="P6" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="Q6" s="5" t="s">
+      <c r="Q6" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="R6" s="5" t="s">
+      <c r="R6" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="S6" s="5" t="s">
+      <c r="S6" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="T6" s="5" t="s">
+      <c r="T6" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="U6" s="5" t="s">
+      <c r="U6" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="V6" s="5" t="s">
+      <c r="V6" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="W6" s="5" t="s">
+      <c r="W6" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="X6" s="5" t="s">
+      <c r="X6" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="Y6" s="5" t="s">
+      <c r="Y6" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="Z6" s="8"/>
-      <c r="AA6" s="8"/>
-      <c r="AB6" s="8"/>
-      <c r="AC6" s="5" t="s">
+      <c r="Z6" s="5"/>
+      <c r="AA6" s="5"/>
+      <c r="AB6" s="5"/>
+      <c r="AC6" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="AD6" s="5" t="s">
+      <c r="AD6" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="AE6" s="5" t="s">
+      <c r="AE6" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="AF6" s="5" t="s">
+      <c r="AF6" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="AG6" s="5" t="s">
+      <c r="AG6" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="AH6" s="5" t="s">
+      <c r="AH6" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="AI6" s="5" t="s">
+      <c r="AI6" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="AJ6" s="5" t="s">
+      <c r="AJ6" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="AK6" s="5" t="s">
+      <c r="AK6" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="AL6" s="5" t="s">
+      <c r="AL6" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="AM6" s="5" t="s">
+      <c r="AM6" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="AN6" s="5" t="s">
+      <c r="AN6" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="AO6" s="5" t="s">
+      <c r="AO6" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="AP6" s="5" t="s">
+      <c r="AP6" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="AQ6" s="5" t="s">
+      <c r="AQ6" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="AR6" s="5" t="s">
+      <c r="AR6" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="AS6" s="5" t="s">
+      <c r="AS6" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="AT6" s="5" t="s">
+      <c r="AT6" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="AU6" s="5" t="s">
+      <c r="AU6" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="AV6" s="5" t="s">
+      <c r="AV6" s="2" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:48" ht="52" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="J7" s="5" t="s">
+      <c r="J7" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="K7" s="5" t="s">
+      <c r="K7" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="L7" s="5" t="s">
+      <c r="L7" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="M7" s="5" t="s">
+      <c r="M7" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="N7" s="5" t="s">
+      <c r="N7" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="O7" s="5" t="s">
+      <c r="O7" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="P7" s="5" t="s">
+      <c r="P7" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="Q7" s="5" t="s">
+      <c r="Q7" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="R7" s="5" t="s">
+      <c r="R7" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="S7" s="5" t="s">
+      <c r="S7" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="T7" s="5" t="s">
+      <c r="T7" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="U7" s="5" t="s">
+      <c r="U7" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="V7" s="5" t="s">
+      <c r="V7" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="W7" s="5" t="s">
+      <c r="W7" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="X7" s="5" t="s">
+      <c r="X7" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="Y7" s="5" t="s">
+      <c r="Y7" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="Z7" s="8"/>
-      <c r="AA7" s="8"/>
-      <c r="AB7" s="8"/>
-      <c r="AC7" s="5" t="s">
+      <c r="Z7" s="5"/>
+      <c r="AA7" s="5"/>
+      <c r="AB7" s="5"/>
+      <c r="AC7" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="AD7" s="5" t="s">
+      <c r="AD7" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="AE7" s="5" t="s">
+      <c r="AE7" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="AF7" s="5" t="s">
+      <c r="AF7" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="AG7" s="5" t="s">
+      <c r="AG7" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="AH7" s="5" t="s">
+      <c r="AH7" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="AI7" s="5" t="s">
+      <c r="AI7" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="AJ7" s="5" t="s">
+      <c r="AJ7" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="AK7" s="5" t="s">
+      <c r="AK7" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AL7" s="5" t="s">
+      <c r="AL7" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AM7" s="5" t="s">
+      <c r="AM7" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="AN7" s="5" t="s">
+      <c r="AN7" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="AO7" s="5" t="s">
+      <c r="AO7" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="AP7" s="5" t="s">
+      <c r="AP7" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="AQ7" s="5" t="s">
+      <c r="AQ7" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="AR7" s="5" t="s">
+      <c r="AR7" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="AS7" s="5" t="s">
+      <c r="AS7" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="AT7" s="5" t="s">
+      <c r="AT7" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="AU7" s="5" t="s">
+      <c r="AU7" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="AV7" s="5" t="s">
+      <c r="AV7" s="2" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="8" spans="1:48" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="9" t="s">
         <v>189</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G8" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="I8" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="J8" s="10" t="s">
+      <c r="J8" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="K8" s="10" t="s">
+      <c r="K8" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="L8" s="10" t="s">
+      <c r="L8" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="M8" s="10" t="s">
+      <c r="M8" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="N8" s="10" t="s">
+      <c r="N8" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="O8" s="10" t="s">
+      <c r="O8" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="P8" s="10" t="s">
+      <c r="P8" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="Q8" s="10" t="s">
+      <c r="Q8" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="R8" s="10" t="s">
+      <c r="R8" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="S8" s="10" t="s">
+      <c r="S8" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="T8" s="10" t="s">
+      <c r="T8" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="U8" s="10" t="s">
+      <c r="U8" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="V8" s="10" t="s">
+      <c r="V8" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="W8" s="10" t="s">
+      <c r="W8" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="X8" s="10" t="s">
+      <c r="X8" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="Y8" s="10" t="s">
+      <c r="Y8" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="Z8" s="9"/>
-      <c r="AA8" s="9"/>
-      <c r="AB8" s="9"/>
-      <c r="AC8" s="10" t="s">
+      <c r="Z8" s="6"/>
+      <c r="AA8" s="6"/>
+      <c r="AB8" s="6"/>
+      <c r="AC8" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="AD8" s="10" t="s">
+      <c r="AD8" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="AE8" s="10" t="s">
+      <c r="AE8" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="AF8" s="10" t="s">
+      <c r="AF8" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="AG8" s="10" t="s">
+      <c r="AG8" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="AH8" s="10" t="s">
+      <c r="AH8" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="AI8" s="10" t="s">
+      <c r="AI8" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="AJ8" s="10" t="s">
+      <c r="AJ8" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="AK8" s="10" t="s">
+      <c r="AK8" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="AL8" s="10" t="s">
+      <c r="AL8" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="AM8" s="10" t="s">
+      <c r="AM8" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="AN8" s="10" t="s">
+      <c r="AN8" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="AO8" s="10" t="s">
+      <c r="AO8" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="AP8" s="10" t="s">
+      <c r="AP8" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="AQ8" s="10" t="s">
+      <c r="AQ8" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="AR8" s="10" t="s">
+      <c r="AR8" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="AS8" s="10" t="s">
+      <c r="AS8" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="AT8" s="10" t="s">
+      <c r="AT8" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="AU8" s="10" t="s">
+      <c r="AU8" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="AV8" s="10" t="s">
+      <c r="AV8" s="3" t="s">
         <v>233</v>
       </c>
     </row>

</xml_diff>